<commit_message>
Added scripts for graphins simulator data and added final report
</commit_message>
<xml_diff>
--- a/data/PlexToGB/5sec_to_1min.xlsx
+++ b/data/PlexToGB/5sec_to_1min.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Jon/usra2026/data/PlexToGB/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{5394672C-91C7-C842-9800-A0FED05445D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ED22B39-E034-034B-91B1-CCDCD10234B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1440" yWindow="500" windowWidth="27320" windowHeight="17500" firstSheet="8" activeTab="16" xr2:uid="{33FA83C0-F142-3742-80B7-FE730F6C474E}"/>
+    <workbookView xWindow="1440" yWindow="500" windowWidth="27320" windowHeight="17500" firstSheet="8" activeTab="10" xr2:uid="{33FA83C0-F142-3742-80B7-FE730F6C474E}"/>
   </bookViews>
   <sheets>
     <sheet name="5sec_morning" sheetId="4" r:id="rId1"/>
@@ -36,112 +36,29 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">allACK!$A$1:$A$309</definedName>
     <definedName name="_xlchart.v1.0" hidden="1">'1min_afternoon'!$K$1:$K$49</definedName>
     <definedName name="_xlchart.v1.1" hidden="1">'20sec_afternon'!$K$1:$K$43</definedName>
-    <definedName name="_xlchart.v1.10" hidden="1">'20sec_afternon'!$K$1:$K$43</definedName>
-    <definedName name="_xlchart.v1.100" hidden="1">total!$B$16</definedName>
-    <definedName name="_xlchart.v1.101" hidden="1">total!$C$16</definedName>
-    <definedName name="_xlchart.v1.102" hidden="1">total!$D$16</definedName>
-    <definedName name="_xlchart.v1.103" hidden="1">total!$E$16</definedName>
-    <definedName name="_xlchart.v1.11" hidden="1">'20sec_afternon'!$K$1:$K$44</definedName>
-    <definedName name="_xlchart.v1.12" hidden="1">'40sec_afternoon'!$K$1:$K$46</definedName>
-    <definedName name="_xlchart.v1.13" hidden="1">'5sec_afternoon'!$K$1:$K$39</definedName>
-    <definedName name="_xlchart.v1.14" hidden="1">total!$B$16</definedName>
-    <definedName name="_xlchart.v1.15" hidden="1">total!$C$16</definedName>
-    <definedName name="_xlchart.v1.16" hidden="1">total!$D$16</definedName>
-    <definedName name="_xlchart.v1.17" hidden="1">total!$E$16</definedName>
-    <definedName name="_xlchart.v1.18" hidden="1">'1min_afternoon'!$K$1:$K$49</definedName>
-    <definedName name="_xlchart.v1.19" hidden="1">'20sec_afternon'!$K$1:$K$43</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">'20sec_afternon'!$K$1:$K$44</definedName>
-    <definedName name="_xlchart.v1.20" hidden="1">'20sec_afternon'!$K$1:$K$44</definedName>
-    <definedName name="_xlchart.v1.21" hidden="1">'40sec_afternoon'!$K$1:$K$46</definedName>
-    <definedName name="_xlchart.v1.22" hidden="1">'5sec_afternoon'!$K$1:$K$39</definedName>
-    <definedName name="_xlchart.v1.23" hidden="1">total!$B$16</definedName>
-    <definedName name="_xlchart.v1.24" hidden="1">total!$C$16</definedName>
-    <definedName name="_xlchart.v1.25" hidden="1">total!$D$16</definedName>
-    <definedName name="_xlchart.v1.26" hidden="1">total!$E$16</definedName>
-    <definedName name="_xlchart.v1.27" hidden="1">'1min_afternoon'!$K$1:$K$49</definedName>
-    <definedName name="_xlchart.v1.28" hidden="1">'20sec_afternon'!$K$1:$K$43</definedName>
-    <definedName name="_xlchart.v1.29" hidden="1">'40sec_afternoon'!$K$1:$K$46</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">'40sec_afternoon'!$K$1:$K$46</definedName>
-    <definedName name="_xlchart.v1.30" hidden="1">total!$C$16</definedName>
-    <definedName name="_xlchart.v1.31" hidden="1">total!$D$16</definedName>
-    <definedName name="_xlchart.v1.32" hidden="1">total!$E$16</definedName>
-    <definedName name="_xlchart.v1.33" hidden="1">total!$AA$33</definedName>
-    <definedName name="_xlchart.v1.34" hidden="1">'1min_afternoon'!$I$1:$I$49</definedName>
-    <definedName name="_xlchart.v1.35" hidden="1">'1min_afternoon'!$K$1:$K$49</definedName>
-    <definedName name="_xlchart.v1.36" hidden="1">'20sec_afternon'!$I$1:$I$43</definedName>
-    <definedName name="_xlchart.v1.37" hidden="1">'20sec_afternon'!$K$1:$K$43</definedName>
-    <definedName name="_xlchart.v1.38" hidden="1">'40sec_afternoon'!$I$1:$I$46</definedName>
-    <definedName name="_xlchart.v1.39" hidden="1">'40sec_afternoon'!$K$1:$K$46</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">'5sec_afternoon'!$K$1:$K$39</definedName>
-    <definedName name="_xlchart.v1.40" hidden="1">'5sec_afternoon'!$I$1:$I$39</definedName>
-    <definedName name="_xlchart.v1.41" hidden="1">total!$B$16</definedName>
-    <definedName name="_xlchart.v1.42" hidden="1">total!$C$16</definedName>
-    <definedName name="_xlchart.v1.43" hidden="1">total!$D$16</definedName>
-    <definedName name="_xlchart.v1.44" hidden="1">total!$E$16</definedName>
-    <definedName name="_xlchart.v1.45" hidden="1">'1min_afternoon'!$K$1:$K$49</definedName>
-    <definedName name="_xlchart.v1.46" hidden="1">'20sec_afternon'!$K$1:$K$43</definedName>
-    <definedName name="_xlchart.v1.47" hidden="1">'20sec_afternon'!$K$1:$K$44</definedName>
-    <definedName name="_xlchart.v1.48" hidden="1">'40sec_afternoon'!$K$1:$K$46</definedName>
-    <definedName name="_xlchart.v1.49" hidden="1">'5sec_afternoon'!$K$1:$K$39</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">total!$B$16</definedName>
-    <definedName name="_xlchart.v1.50" hidden="1">total!$B$16</definedName>
-    <definedName name="_xlchart.v1.51" hidden="1">total!$C$16</definedName>
-    <definedName name="_xlchart.v1.52" hidden="1">total!$D$16</definedName>
-    <definedName name="_xlchart.v1.53" hidden="1">total!$E$16</definedName>
-    <definedName name="_xlchart.v1.54" hidden="1">'1min_afternoon'!$J$1:$J$49</definedName>
-    <definedName name="_xlchart.v1.55" hidden="1">'1min_afternoon'!$K$1:$K$49</definedName>
-    <definedName name="_xlchart.v1.56" hidden="1">'20sec_afternon'!$J$1:$J$43</definedName>
-    <definedName name="_xlchart.v1.57" hidden="1">'20sec_afternon'!$K$1:$K$43</definedName>
-    <definedName name="_xlchart.v1.58" hidden="1">'40sec_afternoon'!$J$1:$J$46</definedName>
-    <definedName name="_xlchart.v1.59" hidden="1">'40sec_afternoon'!$K$1:$K$46</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">total!$C$16</definedName>
-    <definedName name="_xlchart.v1.60" hidden="1">'5sec_afternoon'!$J$1:$J$39</definedName>
-    <definedName name="_xlchart.v1.61" hidden="1">total!$B$16</definedName>
-    <definedName name="_xlchart.v1.62" hidden="1">total!$C$16</definedName>
-    <definedName name="_xlchart.v1.63" hidden="1">total!$D$16</definedName>
-    <definedName name="_xlchart.v1.64" hidden="1">total!$E$16</definedName>
-    <definedName name="_xlchart.v1.65" hidden="1">'1min_afternoon'!$K$1:$K$49</definedName>
-    <definedName name="_xlchart.v1.66" hidden="1">'20sec_afternon'!$K$1:$K$43</definedName>
-    <definedName name="_xlchart.v1.67" hidden="1">'20sec_afternon'!$K$1:$K$44</definedName>
-    <definedName name="_xlchart.v1.68" hidden="1">'40sec_afternoon'!$K$1:$K$46</definedName>
-    <definedName name="_xlchart.v1.69" hidden="1">'5sec_afternoon'!$K$1:$K$39</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">total!$D$16</definedName>
-    <definedName name="_xlchart.v1.70" hidden="1">total!$B$16</definedName>
-    <definedName name="_xlchart.v1.71" hidden="1">total!$C$16</definedName>
-    <definedName name="_xlchart.v1.72" hidden="1">total!$D$16</definedName>
-    <definedName name="_xlchart.v1.73" hidden="1">total!$E$16</definedName>
-    <definedName name="_xlchart.v1.74" hidden="1">'1min_afternoon'!$J$1:$J$49</definedName>
-    <definedName name="_xlchart.v1.75" hidden="1">'1min_afternoon'!$K$1:$K$49</definedName>
-    <definedName name="_xlchart.v1.76" hidden="1">'20sec_afternon'!$J$1:$J$43</definedName>
-    <definedName name="_xlchart.v1.77" hidden="1">'20sec_afternon'!$K$1:$K$43</definedName>
-    <definedName name="_xlchart.v1.78" hidden="1">'40sec_afternoon'!$J$1:$J$46</definedName>
-    <definedName name="_xlchart.v1.79" hidden="1">'40sec_afternoon'!$K$1:$K$46</definedName>
-    <definedName name="_xlchart.v1.8" hidden="1">total!$E$16</definedName>
-    <definedName name="_xlchart.v1.80" hidden="1">'5sec_afternoon'!$J$1:$J$39</definedName>
-    <definedName name="_xlchart.v1.81" hidden="1">total!$B$16</definedName>
-    <definedName name="_xlchart.v1.82" hidden="1">total!$C$16</definedName>
-    <definedName name="_xlchart.v1.83" hidden="1">total!$D$16</definedName>
-    <definedName name="_xlchart.v1.84" hidden="1">total!$E$16</definedName>
-    <definedName name="_xlchart.v1.85" hidden="1">total!$AA$33</definedName>
-    <definedName name="_xlchart.v1.86" hidden="1">'1min_afternoon'!$K$1:$K$49</definedName>
-    <definedName name="_xlchart.v1.87" hidden="1">'20sec_afternon'!$K$1:$K$43</definedName>
-    <definedName name="_xlchart.v1.88" hidden="1">'20sec_afternon'!$K$1:$K$44</definedName>
-    <definedName name="_xlchart.v1.89" hidden="1">'40sec_afternoon'!$K$1:$K$46</definedName>
-    <definedName name="_xlchart.v1.9" hidden="1">'1min_afternoon'!$K$1:$K$49</definedName>
-    <definedName name="_xlchart.v1.90" hidden="1">'5sec_afternoon'!$K$1:$K$39</definedName>
-    <definedName name="_xlchart.v1.91" hidden="1">total!$B$16</definedName>
-    <definedName name="_xlchart.v1.92" hidden="1">total!$C$16</definedName>
-    <definedName name="_xlchart.v1.93" hidden="1">total!$D$16</definedName>
-    <definedName name="_xlchart.v1.94" hidden="1">total!$E$16</definedName>
-    <definedName name="_xlchart.v1.95" hidden="1">'1min_afternoon'!$K$1:$K$49</definedName>
-    <definedName name="_xlchart.v1.96" hidden="1">'20sec_afternon'!$K$1:$K$43</definedName>
-    <definedName name="_xlchart.v1.97" hidden="1">'20sec_afternon'!$K$1:$K$44</definedName>
-    <definedName name="_xlchart.v1.98" hidden="1">'40sec_afternoon'!$K$1:$K$46</definedName>
-    <definedName name="_xlchart.v1.99" hidden="1">'5sec_afternoon'!$K$1:$K$39</definedName>
+    <definedName name="_xlchart.v1.10" hidden="1">total!$B$16</definedName>
+    <definedName name="_xlchart.v1.11" hidden="1">total!$C$16</definedName>
+    <definedName name="_xlchart.v1.12" hidden="1">total!$D$16</definedName>
+    <definedName name="_xlchart.v1.13" hidden="1">total!$E$16</definedName>
+    <definedName name="_xlchart.v1.14" hidden="1">'1min_afternoon'!$J$1:$J$49</definedName>
+    <definedName name="_xlchart.v1.15" hidden="1">'20sec_afternon'!$J$1:$J$43</definedName>
+    <definedName name="_xlchart.v1.16" hidden="1">'40sec_afternoon'!$J$1:$J$46</definedName>
+    <definedName name="_xlchart.v1.17" hidden="1">'5sec_afternoon'!$J$1:$J$39</definedName>
+    <definedName name="_xlchart.v1.18" hidden="1">total!$B$16</definedName>
+    <definedName name="_xlchart.v1.19" hidden="1">total!$C$16</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">'40sec_afternoon'!$K$1:$K$46</definedName>
+    <definedName name="_xlchart.v1.20" hidden="1">total!$D$16</definedName>
+    <definedName name="_xlchart.v1.21" hidden="1">total!$E$16</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">total!$C$16</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">total!$D$16</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">total!$E$16</definedName>
+    <definedName name="_xlchart.v1.6" hidden="1">'1min_afternoon'!$I$1:$I$49</definedName>
+    <definedName name="_xlchart.v1.7" hidden="1">'20sec_afternon'!$I$1:$I$43</definedName>
+    <definedName name="_xlchart.v1.8" hidden="1">'40sec_afternoon'!$I$1:$I$46</definedName>
+    <definedName name="_xlchart.v1.9" hidden="1">'5sec_afternoon'!$I$1:$I$39</definedName>
     <definedName name="_xlnm.Extract" localSheetId="17">allACK!$D:$D</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -6582,17 +6499,17 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.66</cx:f>
+        <cx:f>_xlchart.v1.1</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="1">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.68</cx:f>
+        <cx:f>_xlchart.v1.2</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="2">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.65</cx:f>
+        <cx:f>_xlchart.v1.0</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -6630,7 +6547,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000001-790F-D540-8DB6-3A0F5145A0E8}" formatIdx="1">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.71</cx:f>
+              <cx:f>_xlchart.v1.3</cx:f>
               <cx:v>20sec</cx:v>
             </cx:txData>
           </cx:tx>
@@ -6643,7 +6560,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000000-EC98-A549-A06B-B2C1D324A61C}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.72</cx:f>
+              <cx:f>_xlchart.v1.4</cx:f>
               <cx:v>40sec</cx:v>
             </cx:txData>
           </cx:tx>
@@ -6656,7 +6573,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000001-EC98-A549-A06B-B2C1D324A61C}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.73</cx:f>
+              <cx:f>_xlchart.v1.5</cx:f>
               <cx:v>1min</cx:v>
             </cx:txData>
           </cx:tx>
@@ -6687,22 +6604,22 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.40</cx:f>
+        <cx:f>_xlchart.v1.9</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="1">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.36</cx:f>
+        <cx:f>_xlchart.v1.7</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="2">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.38</cx:f>
+        <cx:f>_xlchart.v1.8</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="3">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.34</cx:f>
+        <cx:f>_xlchart.v1.6</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -6740,7 +6657,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000000-34C6-0042-88D3-7F89D823801D}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.41</cx:f>
+              <cx:f>_xlchart.v1.10</cx:f>
               <cx:v>5sec</cx:v>
             </cx:txData>
           </cx:tx>
@@ -6753,7 +6670,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000001-34C6-0042-88D3-7F89D823801D}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.42</cx:f>
+              <cx:f>_xlchart.v1.11</cx:f>
               <cx:v>20sec</cx:v>
             </cx:txData>
           </cx:tx>
@@ -6766,7 +6683,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000002-34C6-0042-88D3-7F89D823801D}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.43</cx:f>
+              <cx:f>_xlchart.v1.12</cx:f>
               <cx:v>40sec</cx:v>
             </cx:txData>
           </cx:tx>
@@ -6779,7 +6696,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000003-34C6-0042-88D3-7F89D823801D}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.44</cx:f>
+              <cx:f>_xlchart.v1.13</cx:f>
               <cx:v>1min</cx:v>
             </cx:txData>
           </cx:tx>
@@ -6829,22 +6746,22 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.60</cx:f>
+        <cx:f>_xlchart.v1.17</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="1">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.56</cx:f>
+        <cx:f>_xlchart.v1.15</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="2">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.58</cx:f>
+        <cx:f>_xlchart.v1.16</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="3">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.54</cx:f>
+        <cx:f>_xlchart.v1.14</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -6882,7 +6799,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000000-1982-154E-8A89-4170E6163D98}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.61</cx:f>
+              <cx:f>_xlchart.v1.18</cx:f>
               <cx:v>5sec</cx:v>
             </cx:txData>
           </cx:tx>
@@ -6895,7 +6812,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000001-1982-154E-8A89-4170E6163D98}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.62</cx:f>
+              <cx:f>_xlchart.v1.19</cx:f>
               <cx:v>20sec</cx:v>
             </cx:txData>
           </cx:tx>
@@ -6908,7 +6825,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000002-1982-154E-8A89-4170E6163D98}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.63</cx:f>
+              <cx:f>_xlchart.v1.20</cx:f>
               <cx:v>40sec</cx:v>
             </cx:txData>
           </cx:tx>
@@ -6921,7 +6838,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000003-1982-154E-8A89-4170E6163D98}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.64</cx:f>
+              <cx:f>_xlchart.v1.21</cx:f>
               <cx:v>1min</cx:v>
             </cx:txData>
           </cx:tx>
@@ -13904,8 +13821,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="20249552" y="3136718"/>
-              <a:ext cx="4656942" cy="2948982"/>
+              <a:off x="20145298" y="3057106"/>
+              <a:ext cx="4605763" cy="2887378"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -13982,8 +13899,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="24879508" y="3164590"/>
-              <a:ext cx="4641157" cy="2961565"/>
+              <a:off x="24762918" y="3089639"/>
+              <a:ext cx="4604722" cy="2904311"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -14060,8 +13977,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="29418197" y="3122951"/>
-              <a:ext cx="4646430" cy="2961565"/>
+              <a:off x="29265172" y="3048000"/>
+              <a:ext cx="4602709" cy="2904311"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>

</xml_diff>